<commit_message>
(fix) unchangeable amount of ktu and bonus
</commit_message>
<xml_diff>
--- a/bonus_calculator/data/output/output_data.xlsx
+++ b/bonus_calculator/data/output/output_data.xlsx
@@ -92,7 +92,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -317,6 +317,8 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
+    <border/>
     <border/>
     <border/>
     <border/>
@@ -327,7 +329,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -505,6 +507,14 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1188,11 +1198,11 @@
         <v/>
       </c>
       <c r="H11" s="46">
-        <f>ROUND(G11*100/$G$13, 2)</f>
+        <f>100-(SUM(H5:H10)+SUM(H12:H12))</f>
         <v/>
       </c>
       <c r="I11" s="47">
-        <f>ROUND(H11/100*62238.74, 2)</f>
+        <f>62238.74-(SUM(I5:I10)+SUM(I12:I12))</f>
         <v/>
       </c>
     </row>
@@ -1275,14 +1285,14 @@
       <c r="C14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="69" t="inlineStr">
+      <c r="A15" s="73" t="inlineStr">
         <is>
           <t>Премия РП</t>
         </is>
       </c>
       <c r="B15" s="1" t="n"/>
       <c r="C15" s="1" t="n"/>
-      <c r="I15" s="70" t="n">
+      <c r="I15" s="74" t="n">
         <v>14166</v>
       </c>
     </row>

</xml_diff>

<commit_message>
(fix) column A aligment and font
</commit_message>
<xml_diff>
--- a/bonus_calculator/data/output/output_data.xlsx
+++ b/bonus_calculator/data/output/output_data.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="165" formatCode="MMM-YY"/>
     <numFmt numFmtId="166" formatCode="MMM"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <charset val="204"/>
@@ -83,6 +83,10 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -92,7 +96,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="33">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -317,6 +321,8 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
+    <border/>
     <border/>
     <border/>
     <border/>
@@ -329,7 +335,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -516,6 +522,29 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="2"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -898,7 +927,7 @@
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" s="6">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="77" t="inlineStr">
         <is>
           <t>Фактические трудозатраты</t>
         </is>
@@ -913,7 +942,7 @@
       <c r="I2" s="61" t="n"/>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="6">
-      <c r="A3" s="27" t="n"/>
+      <c r="A3" s="78" t="n"/>
       <c r="B3" s="39" t="n">
         <v>2025</v>
       </c>
@@ -932,7 +961,7 @@
       <c r="I3" s="31" t="n"/>
     </row>
     <row r="4" ht="33.75" customHeight="1" s="6">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="78" t="inlineStr">
         <is>
           <t>Ресурсы</t>
         </is>
@@ -967,7 +996,7 @@
       <c r="I4" s="31" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="6">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="78" t="inlineStr">
         <is>
           <t>Тищенко Марина Николаевна</t>
         </is>
@@ -1001,7 +1030,7 @@
       </c>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="78" t="inlineStr">
         <is>
           <t>Ануфриева Оксана Николаевна</t>
         </is>
@@ -1035,7 +1064,7 @@
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="6">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="78" t="inlineStr">
         <is>
           <t>Мирзоян Кристина Владимировна</t>
         </is>
@@ -1069,7 +1098,7 @@
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="6">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="78" t="inlineStr">
         <is>
           <t>Давыдов Артем Васильевич</t>
         </is>
@@ -1104,7 +1133,7 @@
       <c r="J8" s="5" t="n"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="6">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="78" t="inlineStr">
         <is>
           <t>Гапонова Ксения Святославовна</t>
         </is>
@@ -1139,7 +1168,7 @@
       <c r="J9" s="5" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="6">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="78" t="inlineStr">
         <is>
           <t>Никитаев Алексей Вячеславович</t>
         </is>
@@ -1173,7 +1202,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="78" t="inlineStr">
         <is>
           <t>Давлетов Руслан Игоревич</t>
         </is>
@@ -1207,7 +1236,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="inlineStr">
+      <c r="A12" s="79" t="inlineStr">
         <is>
           <t>Харыбин А.В.</t>
         </is>
@@ -1241,7 +1270,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="49" t="inlineStr">
+      <c r="A13" s="79" t="inlineStr">
         <is>
           <t>Общий итог</t>
         </is>
@@ -1280,19 +1309,19 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="n"/>
+      <c r="A14" s="80" t="n"/>
       <c r="B14" s="8" t="n"/>
       <c r="C14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="73" t="inlineStr">
+      <c r="A15" s="81" t="inlineStr">
         <is>
           <t>Премия РП</t>
         </is>
       </c>
       <c r="B15" s="1" t="n"/>
       <c r="C15" s="1" t="n"/>
-      <c r="I15" s="74" t="n">
+      <c r="I15" s="82" t="n">
         <v>14166</v>
       </c>
     </row>
@@ -1310,7 +1339,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n"/>
+      <c r="A17" s="80" t="n"/>
       <c r="B17" s="1" t="n"/>
       <c r="C17" s="1" t="n"/>
     </row>
@@ -1328,7 +1357,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n"/>
+      <c r="A19" s="80" t="n"/>
       <c r="B19" s="3" t="n"/>
       <c r="C19" s="1" t="n"/>
     </row>
@@ -1346,7 +1375,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n"/>
+      <c r="A21" s="80" t="n"/>
       <c r="B21" s="3" t="n"/>
       <c r="C21" s="1" t="n"/>
     </row>
@@ -1363,8 +1392,47 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="83" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="83" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="83" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="83" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="83" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="83" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="83" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="83" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="83" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="83" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="83" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="83" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="83" t="n"/>
+    </row>
     <row r="36">
-      <c r="A36" s="1" t="n"/>
+      <c r="A36" s="80" t="n"/>
       <c r="B36" s="1" t="n"/>
       <c r="C36" s="1" t="n"/>
     </row>

</xml_diff>

<commit_message>
stable version of the reports
</commit_message>
<xml_diff>
--- a/bonus_calculator/data/output/output_data.xlsx
+++ b/bonus_calculator/data/output/output_data.xlsx
@@ -96,7 +96,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -321,6 +321,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
+    <border/>
     <border/>
     <border/>
     <border/>
@@ -335,7 +343,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -545,6 +553,47 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="35" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="36" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="37" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="38" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="39" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="41" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="42" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -886,7 +935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" style="6" min="1" max="1"/>
@@ -998,399 +1047,174 @@
     <row r="5" ht="15.75" customHeight="1" s="6">
       <c r="A5" s="78" t="inlineStr">
         <is>
-          <t>Тищенко Марина Николаевна</t>
+          <t>Гапонова Ксения Святославовна</t>
         </is>
       </c>
       <c r="B5" s="46" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C5" s="46" t="n">
-        <v>145.2595238888889</v>
+        <v>13.14285722222222</v>
       </c>
       <c r="D5" s="46" t="n">
-        <v>101.5</v>
+        <v>30.4</v>
       </c>
       <c r="E5" s="46" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F5" s="46" t="n">
-        <v>2</v>
+        <v>7.5</v>
       </c>
       <c r="G5" s="46">
         <f>ROUND(SUM(B5:F5), 2)</f>
         <v/>
       </c>
-      <c r="H5" s="46">
-        <f>ROUND(G5*100/$G$13, 2)</f>
-        <v/>
-      </c>
-      <c r="I5" s="47">
-        <f>ROUND(H5/100*62238.74, 2)</f>
-        <v/>
+      <c r="H5" s="46" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="I5" s="47" t="n">
+        <v>2414.86</v>
       </c>
     </row>
     <row r="6" ht="31.5" customHeight="1" s="6">
       <c r="A6" s="78" t="inlineStr">
         <is>
-          <t>Ануфриева Оксана Николаевна</t>
-        </is>
-      </c>
-      <c r="B6" s="46" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="C6" s="46" t="n">
-        <v>143.6666666666667</v>
-      </c>
-      <c r="D6" s="46" t="n">
-        <v>98.5</v>
-      </c>
-      <c r="E6" s="46" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="46" t="n">
-        <v>5</v>
+          <t>Общий итог</t>
+        </is>
+      </c>
+      <c r="B6" s="46">
+        <f>ROUND(SUM(B5:B5), 2)</f>
+        <v/>
+      </c>
+      <c r="C6" s="46">
+        <f>ROUND(SUM(C5:C5), 2)</f>
+        <v/>
+      </c>
+      <c r="D6" s="46">
+        <f>ROUND(SUM(D5:D5), 2)</f>
+        <v/>
+      </c>
+      <c r="E6" s="46">
+        <f>ROUND(SUM(E5:E5), 2)</f>
+        <v/>
+      </c>
+      <c r="F6" s="46">
+        <f>ROUND(SUM(F5:F5), 2)</f>
+        <v/>
       </c>
       <c r="G6" s="46">
-        <f>ROUND(SUM(B6:F6), 2)</f>
+        <f>ROUND(SUM(G5:G5), 2)</f>
         <v/>
       </c>
       <c r="H6" s="46">
-        <f>ROUND(G6*100/$G$13, 2)</f>
+        <f>ROUND(SUM(H5:H5), 2)</f>
         <v/>
       </c>
       <c r="I6" s="47">
-        <f>ROUND(H6/100*62238.74, 2)</f>
+        <f>ROUND(SUM(I5:I5), 2)</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="6">
-      <c r="A7" s="78" t="inlineStr">
-        <is>
-          <t>Мирзоян Кристина Владимировна</t>
-        </is>
-      </c>
-      <c r="B7" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="46" t="n">
-        <v>26.92619055555556</v>
-      </c>
-      <c r="D7" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="46">
-        <f>ROUND(SUM(B7:F7), 2)</f>
-        <v/>
-      </c>
-      <c r="H7" s="46">
-        <f>ROUND(G7*100/$G$13, 2)</f>
-        <v/>
-      </c>
-      <c r="I7" s="47">
-        <f>ROUND(H7/100*62238.74, 2)</f>
-        <v/>
-      </c>
+      <c r="A7" s="83" t="n"/>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="6">
-      <c r="A8" s="78" t="inlineStr">
-        <is>
-          <t>Давыдов Артем Васильевич</t>
-        </is>
-      </c>
-      <c r="B8" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="46" t="n">
-        <v>15.59285722222222</v>
-      </c>
-      <c r="D8" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="46">
-        <f>ROUND(SUM(B8:F8), 2)</f>
-        <v/>
-      </c>
-      <c r="H8" s="46">
-        <f>ROUND(G8*100/$G$13, 2)</f>
-        <v/>
-      </c>
-      <c r="I8" s="47">
-        <f>ROUND(H8/100*62238.74, 2)</f>
-        <v/>
-      </c>
-      <c r="J8" s="5" t="n"/>
+      <c r="A8" s="99" t="inlineStr">
+        <is>
+          <t>Премия РП</t>
+        </is>
+      </c>
+      <c r="I8" s="100" t="n">
+        <v>14166</v>
+      </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="6">
-      <c r="A9" s="78" t="inlineStr">
-        <is>
-          <t>Гапонова Ксения Святославовна</t>
-        </is>
-      </c>
-      <c r="B9" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="46" t="n">
-        <v>13.14285722222222</v>
-      </c>
-      <c r="D9" s="46" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="E9" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="46" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G9" s="46">
-        <f>ROUND(SUM(B9:F9), 2)</f>
-        <v/>
-      </c>
-      <c r="H9" s="46">
-        <f>ROUND(G9*100/$G$13, 2)</f>
-        <v/>
-      </c>
-      <c r="I9" s="47">
-        <f>ROUND(H9/100*62238.74, 2)</f>
-        <v/>
-      </c>
-      <c r="J9" s="5" t="n"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Руководитель проекта</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Гапонова К.С.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="6">
-      <c r="A10" s="78" t="inlineStr">
-        <is>
-          <t>Никитаев Алексей Вячеславович</t>
-        </is>
-      </c>
-      <c r="B10" s="46" t="n">
-        <v>20.125</v>
-      </c>
-      <c r="C10" s="46" t="n">
-        <v>130.6761905555556</v>
-      </c>
-      <c r="D10" s="46" t="n">
-        <v>88</v>
-      </c>
-      <c r="E10" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="46">
-        <f>ROUND(SUM(B10:F10), 2)</f>
-        <v/>
-      </c>
-      <c r="H10" s="46">
-        <f>ROUND(G10*100/$G$13, 2)</f>
-        <v/>
-      </c>
-      <c r="I10" s="47">
-        <f>ROUND(H10/100*62238.74, 2)</f>
-        <v/>
-      </c>
+      <c r="A10" s="80" t="n"/>
+      <c r="B10" s="1" t="n"/>
+      <c r="C10" s="1" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="78" t="inlineStr">
-        <is>
-          <t>Давлетов Руслан Игоревич</t>
-        </is>
-      </c>
-      <c r="B11" s="46" t="n">
-        <v>8</v>
-      </c>
-      <c r="C11" s="46" t="n">
-        <v>149.6428572222222</v>
-      </c>
-      <c r="D11" s="46" t="n">
-        <v>136</v>
-      </c>
-      <c r="E11" s="46" t="n">
-        <v>99</v>
-      </c>
-      <c r="F11" s="46" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" s="46">
-        <f>ROUND(SUM(B11:F11), 2)</f>
-        <v/>
-      </c>
-      <c r="H11" s="46">
-        <f>100-(SUM(H5:H10)+SUM(H12:H12))</f>
-        <v/>
-      </c>
-      <c r="I11" s="47">
-        <f>62238.74-(SUM(I5:I10)+SUM(I12:I12))</f>
-        <v/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Куратор / Заказчик</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Амураль И.Б.</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="79" t="inlineStr">
-        <is>
-          <t>Харыбин А.В.</t>
-        </is>
-      </c>
-      <c r="B12" s="48" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="46" t="n">
-        <v>15.59285722222222</v>
-      </c>
-      <c r="D12" s="46" t="n">
-        <v>33</v>
-      </c>
-      <c r="E12" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="46">
-        <f>ROUND(SUM(B12:F12), 2)</f>
-        <v/>
-      </c>
-      <c r="H12" s="46">
-        <f>ROUND(G12*100/$G$13, 2)</f>
-        <v/>
-      </c>
-      <c r="I12" s="47">
-        <f>ROUND(H12/100*62238.74, 2)</f>
-        <v/>
-      </c>
+      <c r="A12" s="80" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="1" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="79" t="inlineStr">
-        <is>
-          <t>Общий итог</t>
-        </is>
-      </c>
-      <c r="B13" s="46">
-        <f>ROUND(SUM(B5:B12), 2)</f>
-        <v/>
-      </c>
-      <c r="C13" s="46">
-        <f>ROUND(SUM(C5:C12), 2)</f>
-        <v/>
-      </c>
-      <c r="D13" s="46">
-        <f>ROUND(SUM(D5:D12), 2)</f>
-        <v/>
-      </c>
-      <c r="E13" s="46">
-        <f>ROUND(SUM(E5:E12), 2)</f>
-        <v/>
-      </c>
-      <c r="F13" s="46">
-        <f>ROUND(SUM(F5:F12), 2)</f>
-        <v/>
-      </c>
-      <c r="G13" s="46">
-        <f>ROUND(SUM(G5:G12), 2)</f>
-        <v/>
-      </c>
-      <c r="H13" s="46">
-        <f>ROUND(SUM(H5:H12), 2)</f>
-        <v/>
-      </c>
-      <c r="I13" s="47">
-        <f>ROUND(SUM(I5:I12), 2)</f>
-        <v/>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Инвестор</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Мегрелишвили М.Э.</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="80" t="n"/>
-      <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
+      <c r="B14" s="3" t="n"/>
+      <c r="C14" s="1" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="81" t="inlineStr">
-        <is>
-          <t>Премия РП</t>
-        </is>
-      </c>
-      <c r="B15" s="1" t="n"/>
-      <c r="C15" s="1" t="n"/>
-      <c r="I15" s="82" t="n">
-        <v>14166</v>
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Руководитель проектного офиса</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Ануфриева О.Н.</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Руководитель проекта</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="1" t="inlineStr">
-        <is>
-          <t>Гапонова К.С.</t>
-        </is>
-      </c>
+      <c r="A16" s="83" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="80" t="n"/>
-      <c r="B17" s="1" t="n"/>
-      <c r="C17" s="1" t="n"/>
+      <c r="A17" s="83" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Куратор / Заказчик</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="1" t="inlineStr">
-        <is>
-          <t>Амураль И.Б.</t>
-        </is>
-      </c>
+      <c r="A18" s="83" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="80" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="1" t="n"/>
+      <c r="A19" s="83" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Инвестор</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>Мегрелишвили М.Э.</t>
-        </is>
-      </c>
+      <c r="A20" s="83" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="80" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="1" t="n"/>
+      <c r="A21" s="83" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Руководитель проектного офиса</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>Ануфриева О.Н.</t>
-        </is>
-      </c>
+      <c r="A22" s="83" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="83" t="n"/>
@@ -1411,30 +1235,9 @@
       <c r="A28" s="83" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="83" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="83" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="83" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="83" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="83" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="83" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="83" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="80" t="n"/>
-      <c r="B36" s="1" t="n"/>
-      <c r="C36" s="1" t="n"/>
+      <c r="A29" s="80" t="n"/>
+      <c r="B29" s="1" t="n"/>
+      <c r="C29" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
(fix) crushed report by changing directory
</commit_message>
<xml_diff>
--- a/bonus_calculator/data/output/output_data.xlsx
+++ b/bonus_calculator/data/output/output_data.xlsx
@@ -96,7 +96,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="44">
+  <borders count="46">
     <border>
       <left/>
       <right/>
@@ -321,6 +321,8 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
+    <border/>
     <border/>
     <border/>
     <border/>
@@ -344,7 +346,7 @@
     <xf numFmtId="44" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
@@ -598,6 +600,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -940,7 +950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" style="6" min="1" max="1"/>
@@ -1084,345 +1094,229 @@
     <row r="6" ht="31.5" customHeight="1" s="6">
       <c r="A6" s="78" t="inlineStr">
         <is>
-          <t>Ануфриева Оксана Николаевна</t>
+          <t>Мирзоян Кристина Владимировна</t>
         </is>
       </c>
       <c r="B6" s="46" t="n">
-        <v>12.5</v>
+        <v>0</v>
       </c>
       <c r="C6" s="46" t="n">
-        <v>143.6666666666667</v>
+        <v>26.92619055555556</v>
       </c>
       <c r="D6" s="46" t="n">
-        <v>98.5</v>
+        <v>0</v>
       </c>
       <c r="E6" s="46" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F6" s="46" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G6" s="46">
         <f>ROUND(SUM(B6:F6), 2)</f>
         <v/>
       </c>
       <c r="H6" s="46" t="n">
-        <v>19.97</v>
+        <v>2.05</v>
       </c>
       <c r="I6" s="47" t="n">
-        <v>12429.08</v>
+        <v>1275.89</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="6">
       <c r="A7" s="78" t="inlineStr">
         <is>
-          <t>Мирзоян Кристина Владимировна</t>
+          <t>Гапонова Ксения Святославовна</t>
         </is>
       </c>
       <c r="B7" s="46" t="n">
         <v>0</v>
       </c>
       <c r="C7" s="46" t="n">
-        <v>26.92619055555556</v>
+        <v>13.14285722222222</v>
       </c>
       <c r="D7" s="46" t="n">
-        <v>0</v>
+        <v>30.4</v>
       </c>
       <c r="E7" s="46" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="46" t="n">
-        <v>0</v>
+        <v>7.5</v>
       </c>
       <c r="G7" s="46">
         <f>ROUND(SUM(B7:F7), 2)</f>
         <v/>
       </c>
       <c r="H7" s="46" t="n">
-        <v>2.05</v>
+        <v>3.88</v>
       </c>
       <c r="I7" s="47" t="n">
-        <v>1275.89</v>
+        <v>2414.86</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="6">
       <c r="A8" s="78" t="inlineStr">
         <is>
-          <t>Давыдов Артем Васильевич</t>
+          <t>Давлетов Руслан Игоревич</t>
         </is>
       </c>
       <c r="B8" s="46" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C8" s="46" t="n">
-        <v>15.59285722222222</v>
+        <v>149.6428572222222</v>
       </c>
       <c r="D8" s="46" t="n">
-        <v>0</v>
+        <v>136</v>
       </c>
       <c r="E8" s="46" t="n">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F8" s="46" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G8" s="46">
         <f>ROUND(SUM(B8:F8), 2)</f>
         <v/>
       </c>
       <c r="H8" s="46" t="n">
-        <v>1.19</v>
+        <v>30.76</v>
       </c>
       <c r="I8" s="47" t="n">
-        <v>740.64</v>
+        <v>19144.64</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="6">
       <c r="A9" s="78" t="inlineStr">
         <is>
-          <t>Гапонова Ксения Святославовна</t>
-        </is>
-      </c>
-      <c r="B9" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="46" t="n">
-        <v>13.14285722222222</v>
-      </c>
-      <c r="D9" s="46" t="n">
-        <v>30.4</v>
-      </c>
-      <c r="E9" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="46" t="n">
-        <v>7.5</v>
+          <t>Общий итог</t>
+        </is>
+      </c>
+      <c r="B9" s="46">
+        <f>ROUND(SUM(B5:B8), 2)</f>
+        <v/>
+      </c>
+      <c r="C9" s="46">
+        <f>ROUND(SUM(C5:C8), 2)</f>
+        <v/>
+      </c>
+      <c r="D9" s="46">
+        <f>ROUND(SUM(D5:D8), 2)</f>
+        <v/>
+      </c>
+      <c r="E9" s="46">
+        <f>ROUND(SUM(E5:E8), 2)</f>
+        <v/>
+      </c>
+      <c r="F9" s="46">
+        <f>ROUND(SUM(F5:F8), 2)</f>
+        <v/>
       </c>
       <c r="G9" s="46">
-        <f>ROUND(SUM(B9:F9), 2)</f>
+        <f>ROUND(SUM(G5:G8), 2)</f>
         <v/>
       </c>
-      <c r="H9" s="46" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="I9" s="47" t="n">
-        <v>2414.86</v>
+      <c r="H9" s="46">
+        <f>ROUND(SUM(H5:H8), 2)</f>
+        <v/>
+      </c>
+      <c r="I9" s="47">
+        <f>ROUND(SUM(I5:I8), 2)</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="6">
-      <c r="A10" s="78" t="inlineStr">
-        <is>
-          <t>Никитаев Алексей Вячеславович</t>
-        </is>
-      </c>
-      <c r="B10" s="46" t="n">
-        <v>20.125</v>
-      </c>
-      <c r="C10" s="46" t="n">
-        <v>130.6761905555556</v>
-      </c>
-      <c r="D10" s="46" t="n">
-        <v>88</v>
-      </c>
-      <c r="E10" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="46">
-        <f>ROUND(SUM(B10:F10), 2)</f>
-        <v/>
-      </c>
-      <c r="H10" s="46" t="n">
-        <v>18.16</v>
-      </c>
-      <c r="I10" s="47" t="n">
-        <v>11302.56</v>
-      </c>
+      <c r="A10" s="83" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="78" t="inlineStr">
-        <is>
-          <t>Давлетов Руслан Игоревич</t>
-        </is>
-      </c>
-      <c r="B11" s="46" t="n">
-        <v>8</v>
-      </c>
-      <c r="C11" s="46" t="n">
-        <v>149.6428572222222</v>
-      </c>
-      <c r="D11" s="46" t="n">
-        <v>136</v>
-      </c>
-      <c r="E11" s="46" t="n">
-        <v>99</v>
-      </c>
-      <c r="F11" s="46" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" s="46">
-        <f>ROUND(SUM(B11:F11), 2)</f>
-        <v/>
-      </c>
-      <c r="H11" s="46" t="n">
-        <v>30.76</v>
-      </c>
-      <c r="I11" s="47" t="n">
-        <v>19144.64</v>
+      <c r="A11" s="105" t="inlineStr">
+        <is>
+          <t>Премия РП</t>
+        </is>
+      </c>
+      <c r="I11" s="106" t="n">
+        <v>14166</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="78" t="inlineStr">
-        <is>
-          <t>Харыбин А.В.</t>
-        </is>
-      </c>
-      <c r="B12" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" s="46" t="n">
-        <v>15.59285722222222</v>
-      </c>
-      <c r="D12" s="46" t="n">
-        <v>33</v>
-      </c>
-      <c r="E12" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="46">
-        <f>ROUND(SUM(B12:F12), 2)</f>
-        <v/>
-      </c>
-      <c r="H12" s="46" t="n">
-        <v>3.7</v>
-      </c>
-      <c r="I12" s="47" t="n">
-        <v>2302.83</v>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Руководитель проекта</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Гапонова К.С.</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="78" t="inlineStr">
-        <is>
-          <t>Общий итог</t>
-        </is>
-      </c>
-      <c r="B13" s="46">
-        <f>ROUND(SUM(B5:B12), 2)</f>
-        <v/>
-      </c>
-      <c r="C13" s="46">
-        <f>ROUND(SUM(C5:C12), 2)</f>
-        <v/>
-      </c>
-      <c r="D13" s="46">
-        <f>ROUND(SUM(D5:D12), 2)</f>
-        <v/>
-      </c>
-      <c r="E13" s="46">
-        <f>ROUND(SUM(E5:E12), 2)</f>
-        <v/>
-      </c>
-      <c r="F13" s="46">
-        <f>ROUND(SUM(F5:F12), 2)</f>
-        <v/>
-      </c>
-      <c r="G13" s="46">
-        <f>ROUND(SUM(G5:G12), 2)</f>
-        <v/>
-      </c>
-      <c r="H13" s="46">
-        <f>ROUND(SUM(H5:H12), 2)</f>
-        <v/>
-      </c>
-      <c r="I13" s="47">
-        <f>ROUND(SUM(I5:I12), 2)</f>
-        <v/>
-      </c>
+      <c r="A13" s="80" t="n"/>
+      <c r="B13" s="1" t="n"/>
+      <c r="C13" s="1" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="83" t="n"/>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Куратор / Заказчик</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Амураль И.Б.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="101" t="inlineStr">
-        <is>
-          <t>Премия РП</t>
-        </is>
-      </c>
-      <c r="I15" s="102" t="n">
-        <v>14166</v>
-      </c>
+      <c r="A15" s="80" t="n"/>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="1" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Руководитель проекта</t>
+          <t>Инвестор</t>
         </is>
       </c>
       <c r="B16" s="2" t="n"/>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>Гапонова К.С.</t>
+          <t>Мегрелишвили М.Э.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="80" t="n"/>
-      <c r="B17" s="1" t="n"/>
+      <c r="B17" s="3" t="n"/>
       <c r="C17" s="1" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Куратор / Заказчик</t>
+          <t>Руководитель проектного офиса</t>
         </is>
       </c>
       <c r="B18" s="2" t="n"/>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>Амураль И.Б.</t>
+          <t>Ануфриева О.Н.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="80" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="1" t="n"/>
+      <c r="A19" s="83" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Инвестор</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>Мегрелишвили М.Э.</t>
-        </is>
-      </c>
+      <c r="A20" s="83" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="80" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="1" t="n"/>
+      <c r="A21" s="83" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Руководитель проектного офиса</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="1" t="inlineStr">
-        <is>
-          <t>Ануфриева О.Н.</t>
-        </is>
-      </c>
+      <c r="A22" s="83" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="83" t="n"/>
@@ -1452,21 +1346,9 @@
       <c r="A31" s="83" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="83" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="83" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="83" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="83" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="80" t="n"/>
-      <c r="B36" s="1" t="n"/>
-      <c r="C36" s="1" t="n"/>
+      <c r="A32" s="80" t="n"/>
+      <c r="B32" s="1" t="n"/>
+      <c r="C32" s="1" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>